<commit_message>
Add columns block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/columns/columns.css
- styles/styles.css
- tools/importer/import-landing-page.bundle.js
- tools/importer/import-landing-page.js
- tools/importer/page-templates.json
- tools/importer/parsers/secure-teasers.js
- tools/importer/reports/ca/en/magazine.report.json
- tools/importer/reports/import-landing-page.report.xlsx
- tools/importer/reports/us/en/magazine.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-landing-page.report.xlsx
+++ b/tools/importer/reports/import-landing-page.report.xlsx
@@ -262,13 +262,13 @@
     <t>ca/en/magazine.report.json</t>
   </si>
   <si>
-    <t>["cards"]</t>
+    <t>["columns","secure-teasers","secure-teasers","cards"]</t>
   </si>
   <si>
     <t>ca/en/magazine</t>
   </si>
   <si>
-    <t>2026-09-09T18:22:53.846Z</t>
+    <t>2026-09-09T19:14:25.327Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -319,7 +319,7 @@
     <t>us/en/magazine</t>
   </si>
   <si>
-    <t>2026-09-09T18:22:47.865Z</t>
+    <t>2026-09-09T19:14:21.177Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine.html</t>

</xml_diff>